<commit_message>
SPM-44, all ACs fulfilled
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-44_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-44_Test_Cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IS212\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D0F036A-7E26-48B6-821F-975829F8EF52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08292416-E44F-4B6A-9808-638B7E494B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" firstSheet="1" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" firstSheet="1" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="167">
   <si>
     <t>Story</t>
   </si>
@@ -183,7 +183,7 @@
     <t>SPM-44-TC10</t>
   </si>
   <si>
-    <t>A confirmed booking cannot be approved over another confirmed booking</t>
+    <t>A pending request cannot be approved over an existing confirmed booking</t>
   </si>
   <si>
     <t>AC6</t>
@@ -583,27 +583,27 @@
     <t>The search screen and the booking check now read the same rule - occupancyConflict() delegates to findVenueConflict(), so the two cannot disagree about whether a room is free.</t>
   </si>
   <si>
-    <t>BLOCKED — there is no way to confirm a booking in the application. Venue Staff's 'Booking Requests' screen lists pending requests but has no Approve or Reject action; that belongs to Venue Booking Approval (SPM-43), which has no endpoint and no branch. The rule itself is implemented and unit tested in src/lib/venueConflict.ts (checkVenueBookingApproval, scope 'approved') — see open question 1.</t>
-  </si>
-  <si>
-    <t>1. Log in as Venue Staff Marcus Wong (marcus.wong@connectsphere.com / password123)
-2. Click 'Booking Requests' in the sidebar
-3. Look for an Approve action on a pending request whose slot another approved booking already holds</t>
-  </si>
-  <si>
-    <t>Blocked pending SPM-43 (Venue Booking Approval)</t>
-  </si>
-  <si>
-    <t>Step 3: No Approve action exists on the screen, so this criterion cannot be exercised through the application. When SPM-43 builds it, approving must be refused with the conflicting booking named, and the unit tests in src/lib/__tests__/venueConflict.test.ts already pin that behaviour.</t>
-  </si>
-  <si>
-    <t>Venue Staff's Booking Requests screen lists pending requests but carries no Approve and no Reject action - zero of each on the page - so there is no way to confirm a booking and the criterion cannot be exercised through the application.</t>
-  </si>
-  <si>
-    <t>Blocked</t>
-  </si>
-  <si>
-    <t>Blocked on SPM-43 (Venue Booking Approval), which has no endpoint and no branch. The rule itself is implemented and unit tested: checkVenueBookingApproval() in src/lib/venueConflict.ts, five tests in venueConflict.test.ts, including that a rival PENDING request must NOT block confirmation. See open question 1.</t>
+    <t>npm run fixtures:spm44 has been run. Two requests exist for SPM44 Conflict Room (SPM44-PLN) on 25 Apr 2027, PM: 'SPM44 Approval Holder' was approved first, and 'SPM44 Approval Rival' is still pending. The pair is seeded rather than made through the app, because the request-time check (SPM-44-TC01) refuses the second request - this is the state Venue Staff inherit when two requests arrive and one is approved. Both events are past approval, so both appear on Booking Requests. Logged in as Venue Staff Marcus Wong (marcus.wong@connectsphere.com / password123).</t>
+  </si>
+  <si>
+    <t>1. Click 'Booking Requests' in the sidebar
+2. Try to click 'Approve' on the 'SPM44 Approval Rival' request</t>
+  </si>
+  <si>
+    <t>Venue: SPM44 Conflict Room (SPM44-PLN), 25 Apr 2027, PM
+Approved first: SPM44 Approval Holder
+Still pending: SPM44 Approval Rival
+Account: marcus.wong@connectsphere.com (Venue Staff)</t>
+  </si>
+  <si>
+    <t>Step 1: The request for 'SPM44 Approval Rival' is listed with the chip 'Conflict' rather than 'Pending', under a panel headed 'This request cannot be approved as it stands' reading 'This overlaps an approved booking: EVT-… SPM44 Approval Holder holds SPM44 Conflict Room on 25 Apr 2027 · PM (13:00–18:00).' with a link to open the calendar.
+Step 2: The Approve button is disabled and nothing happens — the request cannot be confirmed over the booking that already holds the slot. Reject with a reason is still available, which is how Venue Staff clear it.</t>
+  </si>
+  <si>
+    <t>On Venue Staff's Booking Requests screen the 'SPM44 Approval Rival' request is listed with the chip 'Conflict' rather than 'Pending', under a panel headed 'This request cannot be approved as it stands' reading 'This overlaps an approved booking: EVT-001150 SPM44 Approval Holder holds SPM44 Conflict Room on 25 Apr 2027 - PM (13:00-18:00).' with a link to open the calendar. The Approve button is present but disabled; Reject with a reason is still available.</t>
+  </si>
+  <si>
+    <t>Was Blocked until SPM-43 (Review Venue Booking Request) merged to main on 2026-10-04. Merging also settled the duplication SPM-43 had flagged: approvalConflict() carried a second copy of the confirm-time rule and now calls findVenueConflict() with scope 'approved', so a rival PENDING request still does not block a decision. SPM-43's own unit tests pass unchanged, which is the evidence the delegation did not alter behaviour.</t>
   </si>
   <si>
     <t>npm run fixtures:spm44 has been run. Orchard Seminar Room (ORC-SEM) records 60 minutes of setup and 30 of teardown, so a booking there takes one whole adjacent slot either side. 'SPM44 Midnight Holder' holds an APPROVED booking at ORC-SEM on 12 Apr 2027, Night (20:00-22:00) - Night is the last slot of its day, so its turnaround falls on the NEXT day's AM. 'SPM44 Midnight Clash' runs 13 Apr 2027 09:00-11:00 (AM). Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123), assigned to 'SPM44 Midnight Clash'.</t>
@@ -1614,7 +1614,7 @@
         <v>105</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>167</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1656,7 +1656,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="139.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
         <v>88</v>
       </c>
@@ -1664,7 +1664,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
         <v>90</v>
       </c>
@@ -1672,7 +1672,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
         <v>92</v>
       </c>
@@ -1680,7 +1680,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="139.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
         <v>94</v>
       </c>
@@ -1711,7 +1711,7 @@
       <c r="B10" s="5"/>
       <c r="C10" s="6"/>
     </row>
-    <row r="11" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>99</v>
       </c>
@@ -1724,15 +1724,15 @@
         <v>101</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.35">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>103</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
@@ -1740,7 +1740,7 @@
         <v>105</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1787,7 +1787,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.35">
@@ -1795,7 +1795,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.35">
@@ -1803,7 +1803,7 @@
         <v>92</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.35">
@@ -1811,7 +1811,7 @@
         <v>94</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
@@ -1842,7 +1842,7 @@
         <v>99</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
@@ -1858,7 +1858,7 @@
         <v>103</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
@@ -1992,7 +1992,7 @@
         <v>105</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>167</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2118,7 +2118,7 @@
         <v>105</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>97</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2244,7 +2244,7 @@
         <v>105</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2370,7 +2370,7 @@
         <v>105</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>167</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2496,7 +2496,7 @@
         <v>105</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>167</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2622,7 +2622,7 @@
         <v>105</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2748,7 +2748,7 @@
         <v>105</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Docs: import test case workbooks and Sprint 3 regression from Drive
The repo is now the source of truth for test cases. Each SPM-<n>_Test_Cases.xlsx
is replaced by its newer Drive copy, with execution blocks unchanged.
Sprint-3_Regression.xlsx is replaced by the completed run (169 cases,
17-18 Oct 2026). docs/test-cases/README.md covers naming, execution blocks,
retiring a case and when to update the folder.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-44_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-44_Test_Cases.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="176">
   <si>
     <t>Story</t>
   </si>
@@ -391,6 +391,9 @@
     <t>The request is refused with 'SPM44 Conflict Room is already booked for EVT-… SPM44 Approved Holder on 5 Apr 2027, PM.' — naming the event in the way, not just the fact of it. No request is created, and no new row appears under 'Booking requests'.</t>
   </si>
   <si>
+    <t>NA</t>
+  </si>
+  <si>
     <t>Kayalvizhi</t>
   </si>
   <si>
@@ -440,9 +443,6 @@
     <t>With its own pending AM request already in place, SPM44 Conflict Room was still shown as 'Suitable' with a 'Request booking' button on the event's own Venue tab.</t>
   </si>
   <si>
-    <t>NA</t>
-  </si>
-  <si>
     <t>Fail</t>
   </si>
   <si>
@@ -453,6 +453,9 @@
   </si>
   <si>
     <t>Rewritten after review on PR #37 (kayalvizhi24). The earlier version of this case only checked that the button was still shown, and passed on 2026-10-02 - but submitting would have created a second pending request, because the event's own bookings are exempt from the clash check. findDuplicateRequest() now refuses the repeat; two different sessions of one event may still share a room.</t>
+  </si>
+  <si>
+    <t>Janelle Ip</t>
   </si>
   <si>
     <t>npm run fixtures:spm44 has been run. 'SPM44 Pending Holder' holds a PENDING booking request at SPM44 Conflict Room on 6 Apr 2027, PM. 'SPM44 Clash With Pending' runs 6 Apr 2027 14:00-16:00 and has no booking. Logged in as Daniel Tan, assigned to 'SPM44 Clash With Pending'.</t>
@@ -773,7 +776,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -806,32 +809,35 @@
     <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
     <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" vertical="top"/>
@@ -2555,7 +2561,6 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="24.75"/>
     <col customWidth="1" min="2" max="2" width="56.75"/>
-    <col customWidth="1" min="3" max="6" width="12.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -2577,7 +2582,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" ht="84.75" customHeight="1">
@@ -2585,7 +2590,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="5" ht="30.75" customHeight="1">
@@ -2593,7 +2598,7 @@
         <v>92</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" ht="57.75" customHeight="1">
@@ -2601,7 +2606,7 @@
         <v>94</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" ht="17.25" customHeight="1">
@@ -2633,14 +2638,14 @@
         <v>99</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12" ht="17.25" customHeight="1">
       <c r="A12" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -2649,7 +2654,7 @@
         <v>103</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" ht="17.25" customHeight="1">
@@ -2678,13 +2683,15 @@
       <c r="A17" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B17" s="16"/>
+      <c r="B17" s="6" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -2692,21 +2699,23 @@
       <c r="A19" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B19" s="6"/>
+      <c r="B19" s="6" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B20" s="16" t="s">
-        <v>109</v>
+      <c r="B20" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="11">
         <v>46298.0</v>
       </c>
     </row>
@@ -3707,7 +3716,6 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="24.75"/>
     <col customWidth="1" min="2" max="2" width="56.75"/>
-    <col customWidth="1" min="3" max="6" width="12.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -3729,7 +3737,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" ht="71.25" customHeight="1">
@@ -3737,7 +3745,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" ht="17.25" customHeight="1">
@@ -3745,7 +3753,7 @@
         <v>92</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" ht="71.25" customHeight="1">
@@ -3753,7 +3761,7 @@
         <v>94</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" ht="17.25" customHeight="1">
@@ -3785,15 +3793,15 @@
         <v>99</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="12" ht="17.25" customHeight="1">
       <c r="A12" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="17" t="s">
-        <v>166</v>
+      <c r="B12" s="16" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="13" ht="84.75" customHeight="1">
@@ -3801,7 +3809,7 @@
         <v>103</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" ht="17.25" customHeight="1">
@@ -3830,37 +3838,39 @@
       <c r="A17" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B17" s="16"/>
-    </row>
-    <row r="18" ht="15.75" customHeight="1">
+      <c r="B17" s="6" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="18" ht="26.25" customHeight="1">
       <c r="A18" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="16" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1">
+    <row r="19" ht="60.75" customHeight="1">
       <c r="A19" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B19" s="23" t="s">
-        <v>168</v>
+      <c r="B19" s="21" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B20" s="16" t="s">
-        <v>109</v>
+      <c r="B20" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="11">
         <v>46299.0</v>
       </c>
     </row>
@@ -4861,7 +4871,6 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="24.75"/>
     <col customWidth="1" min="2" max="2" width="56.75"/>
-    <col customWidth="1" min="3" max="6" width="12.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -4883,7 +4892,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" ht="84.75" customHeight="1">
@@ -4891,7 +4900,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" ht="84.75" customHeight="1">
@@ -4899,7 +4908,7 @@
         <v>92</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" ht="98.25" customHeight="1">
@@ -4907,7 +4916,7 @@
         <v>94</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7" ht="17.25" customHeight="1">
@@ -4939,14 +4948,14 @@
         <v>99</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="12" ht="17.25" customHeight="1">
       <c r="A12" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -4955,7 +4964,7 @@
         <v>103</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="14" ht="17.25" customHeight="1">
@@ -4984,13 +4993,15 @@
       <c r="A17" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B17" s="16"/>
+      <c r="B17" s="6" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -4998,21 +5009,23 @@
       <c r="A19" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B19" s="6"/>
+      <c r="B19" s="6" t="s">
+        <v>175</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B20" s="16" t="s">
-        <v>109</v>
+      <c r="B20" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="11">
         <v>46298.0</v>
       </c>
     </row>
@@ -6013,7 +6026,6 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="24.75"/>
     <col customWidth="1" min="2" max="2" width="56.75"/>
-    <col customWidth="1" min="3" max="6" width="12.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -6090,7 +6102,7 @@
       <c r="A11" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="6" t="s">
         <v>100</v>
       </c>
     </row>
@@ -6098,7 +6110,7 @@
       <c r="A12" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -6132,11 +6144,11 @@
       </c>
       <c r="B16" s="13"/>
     </row>
-    <row r="17" ht="15.75" customHeight="1">
+    <row r="17" ht="60.75" customHeight="1">
       <c r="A17" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="6" t="s">
         <v>108</v>
       </c>
     </row>
@@ -6144,7 +6156,7 @@
       <c r="A18" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -6152,21 +6164,23 @@
       <c r="A19" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B19" s="6"/>
+      <c r="B19" s="17" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B20" s="16" t="s">
-        <v>109</v>
+      <c r="B20" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="11">
         <v>46298.0</v>
       </c>
     </row>
@@ -7167,7 +7181,6 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="24.75"/>
     <col customWidth="1" min="2" max="2" width="56.75"/>
-    <col customWidth="1" min="3" max="6" width="12.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -7189,7 +7202,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" ht="98.25" customHeight="1">
@@ -7197,7 +7210,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" ht="57.75" customHeight="1">
@@ -7205,7 +7218,7 @@
         <v>92</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" ht="111.75" customHeight="1">
@@ -7213,7 +7226,7 @@
         <v>94</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" ht="17.25" customHeight="1">
@@ -7245,14 +7258,14 @@
         <v>99</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" ht="17.25" customHeight="1">
       <c r="A12" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -7261,7 +7274,7 @@
         <v>103</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" ht="17.25" customHeight="1">
@@ -7291,14 +7304,14 @@
         <v>99</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -7306,21 +7319,23 @@
       <c r="A19" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B19" s="6"/>
+      <c r="B19" s="17" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B20" s="16" t="s">
-        <v>109</v>
+      <c r="B20" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="11">
         <v>46298.0</v>
       </c>
     </row>
@@ -8321,7 +8336,6 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="24.75"/>
     <col customWidth="1" min="2" max="2" width="56.75"/>
-    <col customWidth="1" min="3" max="6" width="12.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -8343,7 +8357,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" ht="71.25" customHeight="1">
@@ -8351,7 +8365,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" ht="30.75" customHeight="1">
@@ -8359,7 +8373,7 @@
         <v>92</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" ht="71.25" customHeight="1">
@@ -8367,7 +8381,7 @@
         <v>94</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" ht="17.25" customHeight="1">
@@ -8399,14 +8413,14 @@
         <v>99</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" ht="17.25" customHeight="1">
       <c r="A12" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -8415,7 +8429,7 @@
         <v>103</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" ht="17.25" customHeight="1">
@@ -8445,14 +8459,14 @@
         <v>99</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="16" t="s">
         <v>122</v>
       </c>
     </row>
@@ -8460,7 +8474,7 @@
       <c r="A19" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="6" t="s">
         <v>123</v>
       </c>
     </row>
@@ -8468,73 +8482,113 @@
       <c r="A20" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B20" s="16" t="s">
-        <v>109</v>
+      <c r="B20" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="11">
         <v>46298.0</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="20" t="s">
+      <c r="A23" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="B23" s="21"/>
+      <c r="B23" s="19"/>
     </row>
     <row r="24" ht="106.5" customHeight="1">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="B24" s="23" t="s">
+      <c r="B24" s="21" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="22" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="22" t="s">
+      <c r="A26" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="B26" s="23" t="s">
+      <c r="B26" s="21" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="B27" s="25" t="s">
+      <c r="B27" s="23" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="22" t="s">
+      <c r="A28" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="B28" s="26">
+      <c r="B28" s="24">
         <v>46301.0</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1"/>
     <row r="30" ht="15.75" customHeight="1"/>
-    <row r="31" ht="15.75" customHeight="1"/>
-    <row r="32" ht="15.75" customHeight="1"/>
-    <row r="33" ht="15.75" customHeight="1"/>
-    <row r="34" ht="15.75" customHeight="1"/>
-    <row r="35" ht="15.75" customHeight="1"/>
-    <row r="36" ht="15.75" customHeight="1"/>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="A31" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="B31" s="19"/>
+    </row>
+    <row r="32" ht="93.75" customHeight="1">
+      <c r="A32" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="B32" s="21" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="B33" s="22" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="34" ht="36.75" customHeight="1">
+      <c r="A34" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="B34" s="25" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="B35" s="26" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="B36" s="27">
+        <v>46303.0</v>
+      </c>
+    </row>
     <row r="37" ht="15.75" customHeight="1"/>
     <row r="38" ht="15.75" customHeight="1"/>
     <row r="39" ht="15.75" customHeight="1"/>
@@ -9517,7 +9571,6 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="24.75"/>
     <col customWidth="1" min="2" max="2" width="56.75"/>
-    <col customWidth="1" min="3" max="6" width="12.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -9539,7 +9592,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" ht="84.75" customHeight="1">
@@ -9547,7 +9600,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" ht="71.25" customHeight="1">
@@ -9555,7 +9608,7 @@
         <v>92</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" ht="57.75" customHeight="1">
@@ -9563,7 +9616,7 @@
         <v>94</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" ht="17.25" customHeight="1">
@@ -9595,14 +9648,14 @@
         <v>99</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" ht="17.25" customHeight="1">
       <c r="A12" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -9611,7 +9664,7 @@
         <v>103</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" ht="17.25" customHeight="1">
@@ -9640,13 +9693,15 @@
       <c r="A17" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B17" s="16"/>
+      <c r="B17" s="6" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -9654,21 +9709,23 @@
       <c r="A19" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B19" s="6"/>
+      <c r="B19" s="6" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B20" s="16" t="s">
-        <v>109</v>
+      <c r="B20" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="11">
         <v>46298.0</v>
       </c>
     </row>
@@ -10669,7 +10726,6 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="24.75"/>
     <col customWidth="1" min="2" max="2" width="56.75"/>
-    <col customWidth="1" min="3" max="6" width="12.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -10691,7 +10747,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" ht="98.25" customHeight="1">
@@ -10699,7 +10755,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" ht="57.75" customHeight="1">
@@ -10707,7 +10763,7 @@
         <v>92</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" ht="71.25" customHeight="1">
@@ -10715,7 +10771,7 @@
         <v>94</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" ht="17.25" customHeight="1">
@@ -10747,14 +10803,14 @@
         <v>99</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="12" ht="17.25" customHeight="1">
       <c r="A12" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -10763,7 +10819,7 @@
         <v>103</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" ht="17.25" customHeight="1">
@@ -10792,13 +10848,15 @@
       <c r="A17" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B17" s="16"/>
+      <c r="B17" s="6" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -10806,21 +10864,23 @@
       <c r="A19" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B19" s="6"/>
+      <c r="B19" s="6" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B20" s="16" t="s">
-        <v>109</v>
+      <c r="B20" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="11">
         <v>46298.0</v>
       </c>
     </row>
@@ -11821,7 +11881,6 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="24.75"/>
     <col customWidth="1" min="2" max="2" width="56.75"/>
-    <col customWidth="1" min="3" max="6" width="12.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -11843,7 +11902,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" ht="98.25" customHeight="1">
@@ -11851,7 +11910,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" ht="57.75" customHeight="1">
@@ -11859,7 +11918,7 @@
         <v>92</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" ht="57.75" customHeight="1">
@@ -11867,7 +11926,7 @@
         <v>94</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" ht="17.25" customHeight="1">
@@ -11899,14 +11958,14 @@
         <v>99</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" ht="17.25" customHeight="1">
       <c r="A12" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -11915,7 +11974,7 @@
         <v>103</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="14" ht="17.25" customHeight="1">
@@ -11944,13 +12003,15 @@
       <c r="A17" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B17" s="16"/>
+      <c r="B17" s="6" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -11958,21 +12019,23 @@
       <c r="A19" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B19" s="6"/>
+      <c r="B19" s="6" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B20" s="16" t="s">
-        <v>109</v>
+      <c r="B20" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="11">
         <v>46298.0</v>
       </c>
     </row>
@@ -12973,7 +13036,6 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="24.75"/>
     <col customWidth="1" min="2" max="2" width="56.75"/>
-    <col customWidth="1" min="3" max="6" width="12.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -12995,7 +13057,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" ht="84.75" customHeight="1">
@@ -13003,7 +13065,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5" ht="71.25" customHeight="1">
@@ -13011,7 +13073,7 @@
         <v>92</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" ht="111.75" customHeight="1">
@@ -13019,7 +13081,7 @@
         <v>94</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" ht="17.25" customHeight="1">
@@ -13051,14 +13113,14 @@
         <v>99</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="12" ht="17.25" customHeight="1">
       <c r="A12" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -13067,7 +13129,7 @@
         <v>103</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14" ht="17.25" customHeight="1">
@@ -13096,13 +13158,15 @@
       <c r="A17" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B17" s="16"/>
+      <c r="B17" s="6" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -13110,21 +13174,23 @@
       <c r="A19" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B19" s="6"/>
+      <c r="B19" s="6" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B20" s="16" t="s">
-        <v>109</v>
+      <c r="B20" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="11">
         <v>46298.0</v>
       </c>
     </row>
@@ -14125,7 +14191,6 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="24.75"/>
     <col customWidth="1" min="2" max="2" width="56.75"/>
-    <col customWidth="1" min="3" max="6" width="12.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -14147,7 +14212,7 @@
         <v>88</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" ht="84.75" customHeight="1">
@@ -14155,7 +14220,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" ht="44.25" customHeight="1">
@@ -14163,7 +14228,7 @@
         <v>92</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" ht="84.75" customHeight="1">
@@ -14171,7 +14236,7 @@
         <v>94</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" ht="17.25" customHeight="1">
@@ -14203,14 +14268,14 @@
         <v>99</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" ht="17.25" customHeight="1">
       <c r="A12" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -14219,7 +14284,7 @@
         <v>103</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="14" ht="17.25" customHeight="1">
@@ -14248,13 +14313,15 @@
       <c r="A17" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B17" s="16"/>
+      <c r="B17" s="6" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -14262,21 +14329,23 @@
       <c r="A19" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B19" s="6"/>
+      <c r="B19" s="6" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B20" s="16" t="s">
-        <v>109</v>
+      <c r="B20" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="11">
         <v>46298.0</v>
       </c>
     </row>

</xml_diff>